<commit_message>
Commiting new changes about range statistics
</commit_message>
<xml_diff>
--- a/bulky_upload_files/correct_freshchat_insights_upoad_template.xlsx
+++ b/bulky_upload_files/correct_freshchat_insights_upoad_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\isadmin\Documents\OMNI-PMS-BACKEND\bulky_upload_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\Omni-projects\OMNI-PMS-BACKEND\bulky_upload_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="35">
   <si>
     <t>user</t>
   </si>
@@ -472,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB11"/>
+  <dimension ref="A1:AB12"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.6640625" style="1" customWidth="1"/>
@@ -583,7 +583,7 @@
     </row>
     <row r="2" spans="1:28" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>26</v>
@@ -595,7 +595,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2" s="1">
         <v>45</v>
@@ -669,7 +669,7 @@
     </row>
     <row r="3" spans="1:28" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>26</v>
@@ -755,7 +755,7 @@
     </row>
     <row r="4" spans="1:28" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>26</v>
@@ -841,7 +841,7 @@
     </row>
     <row r="5" spans="1:28" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>26</v>
@@ -927,7 +927,7 @@
     </row>
     <row r="6" spans="1:28" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>26</v>
@@ -1013,7 +1013,7 @@
     </row>
     <row r="7" spans="1:28" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>26</v>
@@ -1099,7 +1099,7 @@
     </row>
     <row r="8" spans="1:28" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>26</v>
@@ -1111,7 +1111,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F8" s="1">
         <v>56</v>
@@ -1185,7 +1185,7 @@
     </row>
     <row r="9" spans="1:28" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>32</v>
@@ -1197,7 +1197,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="1">
         <v>54</v>
@@ -1271,7 +1271,7 @@
     </row>
     <row r="10" spans="1:28" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>32</v>
@@ -1283,7 +1283,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="1">
         <v>333</v>
@@ -1357,7 +1357,7 @@
     </row>
     <row r="11" spans="1:28" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>32</v>
@@ -1369,7 +1369,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" s="1">
         <v>234</v>
@@ -1438,6 +1438,92 @@
         <v>3</v>
       </c>
       <c r="AB11" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>8</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="1">
+        <v>2</v>
+      </c>
+      <c r="F12" s="1">
+        <v>234</v>
+      </c>
+      <c r="G12" s="1">
+        <v>44</v>
+      </c>
+      <c r="H12" s="1">
+        <v>53</v>
+      </c>
+      <c r="I12" s="1">
+        <v>232</v>
+      </c>
+      <c r="J12" s="1">
+        <v>31</v>
+      </c>
+      <c r="K12" s="1">
+        <v>1</v>
+      </c>
+      <c r="L12" s="1">
+        <v>66</v>
+      </c>
+      <c r="M12" s="1">
+        <v>78</v>
+      </c>
+      <c r="N12" s="1">
+        <v>675</v>
+      </c>
+      <c r="O12" s="1">
+        <v>242</v>
+      </c>
+      <c r="P12" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>66</v>
+      </c>
+      <c r="R12" s="1">
+        <v>1</v>
+      </c>
+      <c r="S12" s="1">
+        <v>4</v>
+      </c>
+      <c r="T12" s="1">
+        <v>6</v>
+      </c>
+      <c r="U12" s="1">
+        <v>75</v>
+      </c>
+      <c r="V12" s="1">
+        <v>32</v>
+      </c>
+      <c r="W12" s="1">
+        <v>453</v>
+      </c>
+      <c r="X12" s="1">
+        <v>73</v>
+      </c>
+      <c r="Y12" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z12" s="1">
+        <v>2</v>
+      </c>
+      <c r="AA12" s="1">
+        <v>3</v>
+      </c>
+      <c r="AB12" s="1" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>